<commit_message>
Update affiliate products database with new lists
</commit_message>
<xml_diff>
--- a/affiliate_data/สัตว์เลี้ยง.xlsx
+++ b/affiliate_data/สัตว์เลี้ยง.xlsx
@@ -442,37 +442,37 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>ยกโหล Nekko อาหารเปียกแมว 70 กรัม12ซอง</v>
+        <v>P&amp;P:กระเป๋าแมว สัตว์เลี้ยง กระเป๋าแมว สุนัข พกกาสัตว์เลีี้ยง สะพายสุนัขและแมวกระเป๋าใส่สัตว์เลี้ยง เดินทางแมว</v>
       </c>
       <c r="C2" t="str">
-        <v>https://down-bs-th.img.susercontent.com/sg-11134201-823r0-mp0pjfpweby84e.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/cn-11134207-7r98o-lykgdbdxz3xefc.webp</v>
       </c>
       <c r="D2" t="str">
-        <v>158.00</v>
+        <v>368.00</v>
       </c>
       <c r="E2" t="str">
         <v/>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>31</v>
       </c>
       <c r="G2" t="str">
-        <v>ขายได้ 5พัน+ ชิ้น</v>
+        <v>ขายได้ 3 ชิ้น</v>
       </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>https://shopee.co.th/product/0/48910813131</v>
+        <v>https://shopee.co.th/product/0/23087897948</v>
       </c>
       <c r="J2" t="str">
-        <v>https://s.shopee.co.th/7AayLy4TAu</v>
+        <v>https://s.shopee.co.th/7VECuLC44H</v>
       </c>
       <c r="K2" t="str">
         <v/>
       </c>
       <c r="L2" t="str">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -480,37 +480,37 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>HYKI - NOTTY Global Version - ห้องน้ำแมวอัตโนมัติ NOTTY by HYKI</v>
+        <v>P&amp;Pกระบะทรายแมวอัตโนมัติ Automatic Cat Toilet ใช้แอพได้ ดีไซน์ใหญ่ รองรับแมวหลายตัว ห้องน้ำแมวอัตโนมัติ ห้องน้ำแมวอัจฉริยะ</v>
       </c>
       <c r="C3" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m4frb6n3mu1683.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/cn-11134207-820l4-mj9k7j7ecbno98.webp</v>
       </c>
       <c r="D3" t="str">
-        <v>7714.00</v>
+        <v>1388.00</v>
       </c>
       <c r="E3" t="str">
         <v/>
       </c>
       <c r="F3" t="str">
-        <v>22</v>
+        <v/>
       </c>
       <c r="G3" t="str">
-        <v>ขายได้ 1พัน+ ชิ้น</v>
+        <v>ขายได้ 12 ชิ้น</v>
       </c>
       <c r="H3" t="str">
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>https://shopee.co.th/product/0/25001294340</v>
+        <v>https://shopee.co.th/product/0/50454380478</v>
       </c>
       <c r="J3" t="str">
-        <v>https://s.shopee.co.th/5L9KAbNLFq</v>
+        <v>https://s.shopee.co.th/5L9iKMTjO5</v>
       </c>
       <c r="K3" t="str">
         <v/>
       </c>
       <c r="L3" t="str">
-        <v>16</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4">
@@ -518,37 +518,37 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>PANDO Pet Dryer Room PD65 แพนโด้ เครื่องเป่าขน สำหรับสัตว์เลี้ยง รุ่น PD65 ตู้เป่าขน อัตโนม</v>
+        <v>ขนมแมว อกไก่ฟรีซดราย 520g ขนมแมวฟรีซดราย 100%ฟู้ดเกรด อกไก่ฟรีซดราย ขนมฟรีซดราย ขนมแมว Freeze dried แมว</v>
       </c>
       <c r="C4" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mp1zyxmcgm4r44.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/th-11134207-7ra0r-mcr6lfk97jyd5f.webp</v>
       </c>
       <c r="D4" t="str">
-        <v>9990.00</v>
+        <v>378.00</v>
       </c>
       <c r="E4" t="str">
         <v/>
       </c>
       <c r="F4" t="str">
-        <v>41</v>
+        <v/>
       </c>
       <c r="G4" t="str">
-        <v>ขายได้ 623 ชิ้น</v>
+        <v>ขายได้ 90 ชิ้น</v>
       </c>
       <c r="H4" t="str">
         <v/>
       </c>
       <c r="I4" t="str">
-        <v>https://shopee.co.th/product/0/24369249453</v>
+        <v>https://shopee.co.th/product/0/29685592246</v>
       </c>
       <c r="J4" t="str">
-        <v>https://s.shopee.co.th/2qRzC0bKNG</v>
+        <v>https://s.shopee.co.th/AUroTrJCmQ</v>
       </c>
       <c r="K4" t="str">
         <v/>
       </c>
       <c r="L4" t="str">
-        <v>5</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5">
@@ -556,37 +556,37 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>F&amp;G วิลล่าแมว Cat Villa บ้านแมว กรงแมว วิลล่าไม้เนื้อแข็งตู้แมว ตู้โชว์ไม้เนื้อแข็ง วิลล่าแมวขนาดใหญ จัดส่งภายใน24ชั่วโม</v>
+        <v>[ประกันศูนย์ไทย] Oneisall Pet Grooming Vacuum Kit 8 in 1 ตัดขนแมว เครื่องดูดขนแมว ไดร์เป่าขนสุนัข ขนาด2.5L รุ่น BM1</v>
       </c>
       <c r="C5" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m3ytl0pibu8a95.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/th-11134207-7ra0h-mdtub2gcu0oe50.webp</v>
       </c>
       <c r="D5" t="str">
-        <v>1999.00</v>
+        <v>5399.00</v>
       </c>
       <c r="E5" t="str">
         <v/>
       </c>
       <c r="F5" t="str">
-        <v>59</v>
+        <v/>
       </c>
       <c r="G5" t="str">
-        <v>ขายได้ 1พัน+ ชิ้น</v>
+        <v>ขายได้ 975 ชิ้น</v>
       </c>
       <c r="H5" t="str">
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>https://shopee.co.th/product/0/22675992236</v>
+        <v>https://shopee.co.th/product/0/26274333150</v>
       </c>
       <c r="J5" t="str">
-        <v>https://s.shopee.co.th/AAEZvUHexi</v>
+        <v>https://s.shopee.co.th/4VabKpijBP</v>
       </c>
       <c r="K5" t="str">
         <v/>
       </c>
       <c r="L5" t="str">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -594,37 +594,37 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>พร้อมส่ง MJ.Kudson อาหารสุนัขพรีเมียมสูตรแกะ (ลดขนร่วง ลดคราบน้ำตา ลดกลิ่นมูลสัตว์) ทานได้ทุกสายพันธุ์</v>
+        <v>P&amp;P:[COD] รังแมว ที่นอนแมว คอกสุนัข เบาะนอนสัตว์เลี้ยง ที่นอนสาน การทอฟาง ซักได้ รังสัตว์เลี้ยง เป็นสากลในทุกฤดูกาลมอบขนมแมวเป็นของขวัญ</v>
       </c>
       <c r="C6" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mopbxox2cfm73f.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/sg-11134201-825zm-mj5axptzj3lva2.webp</v>
       </c>
       <c r="D6" t="str">
-        <v>547.00</v>
+        <v>159.00</v>
       </c>
       <c r="E6" t="str">
         <v/>
       </c>
       <c r="F6" t="str">
-        <v>8</v>
+        <v/>
       </c>
       <c r="G6" t="str">
-        <v>ขายได้ 10พัน+ ชิ้น</v>
+        <v>ขายได้ 75 ชิ้น</v>
       </c>
       <c r="H6" t="str">
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>https://shopee.co.th/product/0/20348607344</v>
+        <v>https://shopee.co.th/product/0/25410281290</v>
       </c>
       <c r="J6" t="str">
-        <v>https://s.shopee.co.th/4AxMmSnMyM</v>
+        <v>https://s.shopee.co.th/2qSNLlyLxx</v>
       </c>
       <c r="K6" t="str">
         <v/>
       </c>
       <c r="L6" t="str">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -632,31 +632,31 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>[🔥ใส่โค้ดลดเพิ่ม] Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรับแมวหลายตัว CATLINK V.3 และ CATLINK V.3 Ultra</v>
+        <v>FABLEME —PET BASKET เข่งใส่แมว ตระกร้าที่นอนแมวแบบเข่ง สไตล์มินิมอลง</v>
       </c>
       <c r="C7" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7ra0k-mbdr25xh8y299a.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/th-11134207-81ztk-mnrcaodqhb0k02.webp</v>
       </c>
       <c r="D7" t="str">
-        <v>13900.00</v>
+        <v>140.00</v>
       </c>
       <c r="E7" t="str">
         <v/>
       </c>
       <c r="F7" t="str">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="G7" t="str">
-        <v>ขายได้ 4พัน+ ชิ้น</v>
+        <v>ขายได้ 64 ชิ้น</v>
       </c>
       <c r="H7" t="str">
         <v/>
       </c>
       <c r="I7" t="str">
-        <v>https://shopee.co.th/product/0/5507071097</v>
+        <v>https://shopee.co.th/product/0/44859868817</v>
       </c>
       <c r="J7" t="str">
-        <v>https://s.shopee.co.th/5fmAZDqFhJ</v>
+        <v>https://s.shopee.co.th/W4SZUGAn5</v>
       </c>
       <c r="K7" t="str">
         <v/>
@@ -670,37 +670,37 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>[ประกันศูนย์ไทย] Oneisall Pet Grooming Vacuum Kit 8 in 1 ตัดขนแมว เครื่องดูดขนแมว ไดร์เป่าขนสุนัข ขนาด2.5L รุ่น BM1</v>
+        <v>Whiskas® วิสกัส อาหารเม็ดสำหรับแมว ขนาด 1.1 - 1.2 kg</v>
       </c>
       <c r="C8" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7ra0h-mdtub2gcu0oe50.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/th-11134207-7ras9-m3q7953p6s4o6e.webp</v>
       </c>
       <c r="D8" t="str">
-        <v>5372.00</v>
+        <v>159.00</v>
       </c>
       <c r="E8" t="str">
         <v/>
       </c>
       <c r="F8" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="G8" t="str">
-        <v>ขายได้ 963 ชิ้น</v>
+        <v>ขายได้ 3พัน+ ชิ้น</v>
       </c>
       <c r="H8" t="str">
         <v/>
       </c>
       <c r="I8" t="str">
-        <v>https://shopee.co.th/product/0/26274333150</v>
+        <v>https://shopee.co.th/product/0/26170558021</v>
       </c>
       <c r="J8" t="str">
-        <v>https://s.shopee.co.th/3qKWNr61yu</v>
+        <v>https://s.shopee.co.th/AAEy5FpGxh</v>
       </c>
       <c r="K8" t="str">
         <v/>
       </c>
       <c r="L8" t="str">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -708,37 +708,37 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>Petology คอนโดแมวคุณภาพสูง แข็งแรง ทนทาน ใช้งานได้นาน รุ่น CD-01</v>
+        <v>Dr.Zkin Pet Spray ผลิตภัณฑ์สำหรับสัตว์เลี้ยง บำรุงขน ดับกลิ่น เพิ่มความหอม</v>
       </c>
       <c r="C9" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7ra0i-mbdqw6sm2nna5d.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/th-11134207-81ztg-mhh7zikraarne4.webp</v>
       </c>
       <c r="D9" t="str">
-        <v>11000.00</v>
+        <v>210.00</v>
       </c>
       <c r="E9" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v/>
+        <v>55</v>
       </c>
       <c r="G9" t="str">
-        <v>ขายได้ 151 ชิ้น</v>
+        <v>ขายได้ 2พัน+ ชิ้น</v>
       </c>
       <c r="H9" t="str">
         <v/>
       </c>
       <c r="I9" t="str">
-        <v>https://shopee.co.th/product/0/6331670112</v>
+        <v>https://shopee.co.th/product/0/25456988939</v>
       </c>
       <c r="J9" t="str">
-        <v>https://s.shopee.co.th/40dwaAECCx</v>
+        <v>https://s.shopee.co.th/6VLfiWAAsM</v>
       </c>
       <c r="K9" t="str">
         <v/>
       </c>
       <c r="L9" t="str">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -746,37 +746,37 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>[เลือกรสชาติได้] Purina ONE อาหารแมว 10 kg</v>
+        <v>P&amp;P:ให้คุกกี้แมวบ้านแมวโดนัท อุโมงค์แมว ของเล่นแมว ที่นอนแมว วัสดุแข็งแรงที่นอนแมว ของเล่นแมว</v>
       </c>
       <c r="C10" t="str">
-        <v>https://down-bs-th.img.susercontent.com/sg-11134201-823ok-mp3h99k9jb4c65.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/cn-11134207-820l4-mjia39ghxcslf6.webp</v>
       </c>
       <c r="D10" t="str">
-        <v>1499.00</v>
+        <v>400.00</v>
       </c>
       <c r="E10" t="str">
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>16</v>
+        <v/>
       </c>
       <c r="G10" t="str">
-        <v>ขายได้ 10พัน+ ชิ้น</v>
+        <v>ขายได้ 1พัน+ ชิ้น</v>
       </c>
       <c r="H10" t="str">
         <v/>
       </c>
       <c r="I10" t="str">
-        <v>https://shopee.co.th/product/0/42922380987</v>
+        <v>https://shopee.co.th/product/0/16595556490</v>
       </c>
       <c r="J10" t="str">
-        <v>https://s.shopee.co.th/8ATVXp85zW</v>
+        <v>https://s.shopee.co.th/9AMQtQDq9g</v>
       </c>
       <c r="K10" t="str">
         <v/>
       </c>
       <c r="L10" t="str">
-        <v>7</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11">
@@ -784,13 +784,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>BIO น้ำยาดับกลิ่น กลิ่นฉี่ กลิ่นมูลสัตว์เลี้ยง ล้างพื้นกลิ่นฉี่ ทำความสะอาด ปราศจากเชื้อโรค กลิ่นโอโซนบริสุทธิ์ 1,000 ml</v>
+        <v>P＆P:ทรายแมวผสม 4ลิตร ออร์แกนิค100% อัตราส่วนพิเศษ มีประสิทธิภาพในการกำจัดกลิ่นเหม็น ทรายแมว ทรายเต้าหู้ ทรายเบนโทไนท์</v>
       </c>
       <c r="C11" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7r98x-lopnhfgn1k599e.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/cn-11134207-820l4-milf64oo84cg40.webp</v>
       </c>
       <c r="D11" t="str">
-        <v>209.00</v>
+        <v>216.00</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -799,22 +799,22 @@
         <v/>
       </c>
       <c r="G11" t="str">
-        <v>ขายได้ 5พัน+ ชิ้น</v>
+        <v>ขายได้ 270 ชิ้น</v>
       </c>
       <c r="H11" t="str">
         <v/>
       </c>
       <c r="I11" t="str">
-        <v>https://shopee.co.th/product/0/25452334947</v>
+        <v>https://shopee.co.th/product/0/26658414705</v>
       </c>
       <c r="J11" t="str">
-        <v>https://s.shopee.co.th/8V6LwRFcsS</v>
+        <v>https://s.shopee.co.th/8ATthaQaH8</v>
       </c>
       <c r="K11" t="str">
         <v/>
       </c>
       <c r="L11" t="str">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12">
@@ -822,37 +822,37 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>Dr.Zkin Pet Spray ผลิตภัณฑ์สำหรับสัตว์เลี้ยง บำรุงขน ดับกลิ่น เพิ่มความหอม</v>
+        <v>Kaniva Urinary Care อาหารแมว ดูแลทางเดินปัสสาวะ แมว 4 เดือนขึ้นไป Petus Kingkaew</v>
       </c>
       <c r="C12" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mhh7zikraarne4.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/th-11134207-81ztl-mnjve9j6jp4w53.webp</v>
       </c>
       <c r="D12" t="str">
-        <v>210.00</v>
+        <v>799.00</v>
       </c>
       <c r="E12" t="str">
         <v/>
       </c>
       <c r="F12" t="str">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="G12" t="str">
-        <v>ขายได้ 2พัน+ ชิ้น</v>
+        <v>ขายได้ 24 ชิ้น</v>
       </c>
       <c r="H12" t="str">
         <v/>
       </c>
       <c r="I12" t="str">
-        <v>https://shopee.co.th/product/0/25456988939</v>
+        <v>https://shopee.co.th/product/0/24543543686</v>
       </c>
       <c r="J12" t="str">
-        <v>https://s.shopee.co.th/70HY9gQhNc</v>
+        <v>https://s.shopee.co.th/1BK9MizH9w</v>
       </c>
       <c r="K12" t="str">
         <v/>
       </c>
       <c r="L12" t="str">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -860,13 +860,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>บ้านน็อคดาวน์ สำเร็จรูป</v>
+        <v>Jaotoob ทิชชู่เปียกสัตว์เลี้ยง สูตรสปาอ่อนโยน กลิ่น Dreamy Spa | 80 แผ่น หนานุ่ม ขนาดใหญ่ 20×20 ซม.</v>
       </c>
       <c r="C13" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-m7wxzwgmmrgc2f.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/th-11134207-81zto-mla2wh5ox7gka3.webp</v>
       </c>
       <c r="D13" t="str">
-        <v>150000.00</v>
+        <v>189.00</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -875,22 +875,22 @@
         <v/>
       </c>
       <c r="G13" t="str">
-        <v/>
+        <v>ขายได้ 560 ชิ้น</v>
       </c>
       <c r="H13" t="str">
         <v/>
       </c>
       <c r="I13" t="str">
-        <v>https://shopee.co.th/product/0/25993261993</v>
+        <v>https://shopee.co.th/product/0/40977662998</v>
       </c>
       <c r="J13" t="str">
-        <v>https://s.shopee.co.th/30lPOKnQ4s</v>
+        <v>https://s.shopee.co.th/4AxkwExCja</v>
       </c>
       <c r="K13" t="str">
         <v/>
       </c>
       <c r="L13" t="str">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
@@ -898,37 +898,37 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>Prowild โปรไวลด์ ซีเล็คเต็ด อาหารสุนัขทุกสายพันธุ์/ทุกช่วงวัย ขนาด 15 kg</v>
+        <v>คอนโดแมว ที่รับเล็บแมว กรอบปีนแมว เสาลับเล็บแมวได้ แคปซูลอวกาศ รางบอลแมว ทนต่อการขีดข่วน</v>
       </c>
       <c r="C14" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7ra0m-mbg6gn8vi82g66.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/sg-11134201-820md-mnctgoxnur5y17.webp</v>
       </c>
       <c r="D14" t="str">
-        <v>1590.00</v>
+        <v>228.00</v>
       </c>
       <c r="E14" t="str">
         <v/>
       </c>
       <c r="F14" t="str">
-        <v/>
+        <v>71</v>
       </c>
       <c r="G14" t="str">
-        <v>ขายได้ 30พัน+ ชิ้น</v>
+        <v>ขายได้ 3พัน+ ชิ้น</v>
       </c>
       <c r="H14" t="str">
         <v/>
       </c>
       <c r="I14" t="str">
-        <v>https://shopee.co.th/product/0/3670154648</v>
+        <v>https://shopee.co.th/product/0/42280293068</v>
       </c>
       <c r="J14" t="str">
-        <v>https://s.shopee.co.th/9fIJKaWMHK</v>
+        <v>https://s.shopee.co.th/4VabKr5hIH</v>
       </c>
       <c r="K14" t="str">
         <v/>
       </c>
       <c r="L14" t="str">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -936,13 +936,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรับแมวหลายตัว CATLINK Lite</v>
+        <v>🐈🐱Neakasa M1 2024 ห้องน้ำแมวอัตโนมัติ I Smart Cat Litter I จัดการข้อมูลแมว 3 ตัว I แอปควบคุมระยะไกล🐈🐱</v>
       </c>
       <c r="C15" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7ras9-mauvmoz6b0omd5.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/th-11134207-7rasi-m6oxwve9ydkf40.webp</v>
       </c>
       <c r="D15" t="str">
-        <v>8800.00</v>
+        <v>11800.00</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -951,22 +951,22 @@
         <v/>
       </c>
       <c r="G15" t="str">
-        <v>ขายได้ 2พัน+ ชิ้น</v>
+        <v>ขายได้ 839 ชิ้น</v>
       </c>
       <c r="H15" t="str">
         <v/>
       </c>
       <c r="I15" t="str">
-        <v>https://shopee.co.th/product/0/8904141232</v>
+        <v>https://shopee.co.th/product/0/27771402652</v>
       </c>
       <c r="J15" t="str">
-        <v>https://s.shopee.co.th/60P0xquu84</v>
+        <v>https://s.shopee.co.th/9zvXsxsJyp</v>
       </c>
       <c r="K15" t="str">
         <v/>
       </c>
       <c r="L15" t="str">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -974,37 +974,37 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>แมว ไดร์เป่าผม 62 /82L ของใช้แมว เครื่องเป่าขนแมว อาบน้ําแมว ตู้อบแมว ตั้งเวลาได้ ไดร์เป่าขนแมว</v>
+        <v>whiskas วิสกัส อาหารแมว ลูกแมว แมวโต 1.1-1.2 กก</v>
       </c>
       <c r="C16" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134201-7rasf-maxkg8lg2suo1b.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/th-11134207-81zti-mf6g50dtqy3183.webp</v>
       </c>
       <c r="D16" t="str">
-        <v>2933.00</v>
+        <v>155.00</v>
       </c>
       <c r="E16" t="str">
         <v/>
       </c>
       <c r="F16" t="str">
-        <v>51</v>
+        <v/>
       </c>
       <c r="G16" t="str">
-        <v>ขายได้ 193 ชิ้น</v>
+        <v>ขายได้ 85 ชิ้น</v>
       </c>
       <c r="H16" t="str">
         <v/>
       </c>
       <c r="I16" t="str">
-        <v>https://shopee.co.th/product/0/29425138487</v>
+        <v>https://shopee.co.th/product/0/25986964321</v>
       </c>
       <c r="J16" t="str">
-        <v>https://s.shopee.co.th/9fIJKasq1a</v>
+        <v>https://s.shopee.co.th/6AipJvFRH4</v>
       </c>
       <c r="K16" t="str">
         <v/>
       </c>
       <c r="L16" t="str">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17">
@@ -1012,37 +1012,37 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>คอกกระบะฮันเตอร์(Hunter Cage)</v>
+        <v>นาโนพาวเวอร์ ทิชชู่เปียกซิลเวอร์นาโน ทำความสะอาดและทรีทเม้นต์บำรุงสำหรับสัตว์เลี้ยง (100 แผ่น)</v>
       </c>
       <c r="C17" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7qul0-lfgefx1hi2su42.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/th-11134207-81zte-mnfp1sbrpaf79a.webp</v>
       </c>
       <c r="D17" t="str">
-        <v>11715.00</v>
+        <v>175.00</v>
       </c>
       <c r="E17" t="str">
         <v/>
       </c>
       <c r="F17" t="str">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G17" t="str">
-        <v>ขายได้ 343 ชิ้น</v>
+        <v>ขายได้ 2พัน+ ชิ้น</v>
       </c>
       <c r="H17" t="str">
         <v/>
       </c>
       <c r="I17" t="str">
-        <v>https://shopee.co.th/product/0/20378259987</v>
+        <v>https://shopee.co.th/product/0/12202164414</v>
       </c>
       <c r="J17" t="str">
-        <v>https://s.shopee.co.th/gNUc3Zcns</v>
+        <v>https://s.shopee.co.th/9UzHI3D3qU</v>
       </c>
       <c r="K17" t="str">
         <v/>
       </c>
       <c r="L17" t="str">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18">
@@ -1050,31 +1050,31 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>[เลือกรสชาติได้] Purina One อาหารแมว 6.6กก</v>
+        <v>Mango 2 IN 1 เก้าอี้ลับเล็บแมว เก้าอี้แมว+เสื่อ เสื่อลับเล็บ ไม่เป็นขุย เปลญวนแมว โซฟาลับเล็บ เตียงแมว โซฟาแมว</v>
       </c>
       <c r="C18" t="str">
-        <v>https://down-bs-th.img.susercontent.com/sg-11134201-823rm-mp2iqoc9yo7jc3.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/sg-11134201-81zwi-mn29u65vzpqa69.webp</v>
       </c>
       <c r="D18" t="str">
-        <v>1149.00</v>
+        <v>122.00</v>
       </c>
       <c r="E18" t="str">
         <v/>
       </c>
       <c r="F18" t="str">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="G18" t="str">
-        <v>ขายได้ 40พัน+ ชิ้น</v>
+        <v>ขายได้ 98 ชิ้น</v>
       </c>
       <c r="H18" t="str">
         <v/>
       </c>
       <c r="I18" t="str">
-        <v>https://shopee.co.th/product/0/10998396488</v>
+        <v>https://shopee.co.th/product/0/46708865917</v>
       </c>
       <c r="J18" t="str">
-        <v>https://s.shopee.co.th/2LVib7bsCQ</v>
+        <v>https://s.shopee.co.th/110jAQnCXd</v>
       </c>
       <c r="K18" t="str">
         <v/>
@@ -1088,37 +1088,37 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>🐈🐱Neakasa M1 2024 ห้องน้ำแมวอัตโนมัติ I Smart Cat Litter I จัดการข้อมูลแมว 3 ตัว I แอปควบคุมระยะไกล🐈🐱</v>
+        <v>HYKI - NOTTY Global Version - ห้องน้ำแมวอัตโนมัติ NOTTY by HYKI</v>
       </c>
       <c r="C19" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7rasi-m6oxwve9ydkf40.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/th-11134207-7rasm-m4frb6n3mu1683.webp</v>
       </c>
       <c r="D19" t="str">
-        <v>10499.00</v>
+        <v>7722.00</v>
       </c>
       <c r="E19" t="str">
         <v/>
       </c>
       <c r="F19" t="str">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="G19" t="str">
-        <v>ขายได้ 835 ชิ้น</v>
+        <v>ขายได้ 1พัน+ ชิ้น</v>
       </c>
       <c r="H19" t="str">
         <v/>
       </c>
       <c r="I19" t="str">
-        <v>https://shopee.co.th/product/0/27771402652</v>
+        <v>https://shopee.co.th/product/0/25001294340</v>
       </c>
       <c r="J19" t="str">
-        <v>https://s.shopee.co.th/8V6LwSP3Kc</v>
+        <v>https://s.shopee.co.th/6L2FWEcevl</v>
       </c>
       <c r="K19" t="str">
         <v/>
       </c>
       <c r="L19" t="str">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20">
@@ -1126,13 +1126,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>Petoya คอลลาเจนญี่ปุ่นบำรุงข้อและขน สำหรับสุนัขและแมว สูตร Joint Focus + DHA</v>
+        <v>Pramy Carnivore (พรามี่ คาร์นิวอร์) อาหารเปียกแมว มีให้เลือก 8 สูตร (70g.*12ซอง)</v>
       </c>
       <c r="C20" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7r98s-lxa2x1xegij3c3.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/th-11134207-7r98z-lzdfjwhwr0xtad.webp</v>
       </c>
       <c r="D20" t="str">
-        <v>490.00</v>
+        <v>215.00</v>
       </c>
       <c r="E20" t="str">
         <v/>
@@ -1141,22 +1141,22 @@
         <v/>
       </c>
       <c r="G20" t="str">
-        <v>ขายได้ 3พัน+ ชิ้น</v>
+        <v>ขายได้ 5พัน+ ชิ้น</v>
       </c>
       <c r="H20" t="str">
         <v/>
       </c>
       <c r="I20" t="str">
-        <v>https://shopee.co.th/product/0/18483804394</v>
+        <v>https://shopee.co.th/product/0/28509086464</v>
       </c>
       <c r="J20" t="str">
-        <v>https://s.shopee.co.th/6py7xOYUW1</v>
+        <v>https://s.shopee.co.th/2qSNLnxTd1</v>
       </c>
       <c r="K20" t="str">
         <v/>
       </c>
       <c r="L20" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -1164,37 +1164,37 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>กรงไก่กลางแจ้ง คอกไก่ บ้านไก่ ขนาดใหญ่พิเศษ สำหรับการเลี้ยงสัตว์ปีก กันฝน กรงนกยูงและนกพิราบ โครงสร้างขนาดใหญ่</v>
+        <v>P&amp;P:โปรไบโอติกสำหรับสัตว์เลี้ยง วิตามินหมา วิตามินแมว โปรไบโอติค เสริมภูมิ บำรุงขน สำหรับสุนัขและแมว บำรุงขนผิว ช่วยให้เจริญอาหาร 180 แคปซูลมอบขนมแมวเป็นของขวัญ</v>
       </c>
       <c r="C21" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mkdbuy6rdgjr2e.webp</v>
+        <v>https://down-zl-th.img.susercontent.com/cn-11134207-820l4-mj5augmdo7b4ac.webp</v>
       </c>
       <c r="D21" t="str">
-        <v>1186.00</v>
+        <v>133.00</v>
       </c>
       <c r="E21" t="str">
         <v/>
       </c>
       <c r="F21" t="str">
-        <v>27</v>
+        <v/>
       </c>
       <c r="G21" t="str">
-        <v>ขายได้ 198 ชิ้น</v>
+        <v>ขายได้ 206 ชิ้น</v>
       </c>
       <c r="H21" t="str">
         <v/>
       </c>
       <c r="I21" t="str">
-        <v>https://shopee.co.th/product/0/51205882798</v>
+        <v>https://shopee.co.th/product/0/20686812352</v>
       </c>
       <c r="J21" t="str">
-        <v>https://s.shopee.co.th/8Kmvk9b1wJ</v>
+        <v>https://s.shopee.co.th/BRcAuHjaM</v>
       </c>
       <c r="K21" t="str">
         <v/>
       </c>
       <c r="L21" t="str">
-        <v>7</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>